<commit_message>
Attribute Cool Places listings to their real bookable providers
Cool Places is an enquiry-only aggregator, so each of its 43 listings is re-mapped to its actual bookable source (Independent Cottages, Host Unusual, Coolstays, Sykes, Champing, St Hilda, etc.) via new 'Source provider'/'Original source link' columns. build_data.py honours a per-row provider_col and still groups 'featured' by the originating sheet so the homepage isn't flooded. 28 providers now; 'Cool Places' no longer shown as a provider; all listing links resolve. Unified 0-100 scores incl. the fairness adjustment are unchanged (Hafod 67, Henry 82).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CoolPlaces_digitaldetox_remoteness_ranking.xlsx
+++ b/data/CoolPlaces_digitaldetox_remoteness_ranking.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -604,6 +604,16 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Full-size image URLs (array)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Source provider</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Original source link</t>
         </is>
       </c>
     </row>
@@ -695,6 +705,16 @@
 https://assets.coolplaces.co.uk/images/843d9385076521b1af9fe0c671d6ff4d2dc645ea/large.jpg</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Solomon's Island</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>https://solomonsisland.co.uk/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -766,6 +786,16 @@
 https://assets.coolplaces.co.uk/images/a18a68eae08c7a3a6dcd4b87fdf4feb6c26f6e2f/large.jpg
 https://assets.coolplaces.co.uk/images/b61195f8b0099a0dd99d3b68504a72d98aa66f57/large.jpg
 https://assets.coolplaces.co.uk/images/a432ef3a319cb0063a06fe1ab2af81100435a549/large.jpg</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>YHA</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>https://www.yha.org.uk/hostel/yha-black-sail</t>
         </is>
       </c>
     </row>
@@ -848,6 +878,16 @@
 https://assets.coolplaces.co.uk/images/2e037bc0a7b06b2cd9ee6696b57b08431b60f62c/large.jpg</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Ardnish</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>https://www.ardnish.org/bothy/booking.php</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -925,6 +965,16 @@
 https://assets.coolplaces.co.uk/images/9189ade060d2bc9297cb01539541dbc07a0247ea/large.jpg
 https://assets.coolplaces.co.uk/images/1dbc1ab50da558d19661db51634422506d09e476/large.jpg
 https://assets.coolplaces.co.uk/images/3d2aa638d4670785c34736b1aba20e623e799447/large.jpg</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Independent Cottages</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>https://www.independentcottages.co.uk/highland/laggan-ref3136</t>
         </is>
       </c>
     </row>
@@ -1011,6 +1061,16 @@
 https://assets.coolplaces.co.uk/images/f3e92fe89b06feb74b2f30ff82ee7d6fac4243bd/large.jpg
 https://assets.coolplaces.co.uk/images/788d58cedae66a0dcc9bf2bf1f7220cf34804569/large.jpg
 https://assets.coolplaces.co.uk/images/000060ae3d60bb5129ed39b2a56b8bdca67dfa19/large.jpg</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Independent Cottages</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>https://www.independentcottages.co.uk/highland/lower-polnish-ref3696</t>
         </is>
       </c>
     </row>
@@ -1108,6 +1168,16 @@
 https://assets.coolplaces.co.uk/images/a1a2c2943a0f09423796c81f710d8e168d4d10f4/large.jpg</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/the-linhay/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1189,6 +1259,16 @@
 https://assets.coolplaces.co.uk/images/8a2fee7831d331a24942c9ecf2ffcbc6c73d29c7/large.jpg
 https://assets.coolplaces.co.uk/images/e4af08e7265d2a404a0e6397fe94b44eab997047/large.jpg
 https://assets.coolplaces.co.uk/images/8b94078dd7ea3e0b4c8e65652a0a1630c82d897b/large.jpg</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>St Hilda Sea Adventures</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>https://www.sthildaseaadventures.co.uk/</t>
         </is>
       </c>
     </row>
@@ -1275,6 +1355,16 @@
 https://assets.coolplaces.co.uk/images/c4249816061b1fffb202e3e48822f7f5e09846dd/large.jpg</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Coolstays</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>https://www.coolstays.com/property/the-boathouse-at-knotts-end/19883</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1355,6 +1445,16 @@
 https://assets.coolplaces.co.uk/images/1ecf57467442eb0db3811079f8a8d166847c4cd4/large.jpg
 https://assets.coolplaces.co.uk/images/6f3d76a812caf9fbde16c77ce4fd6ad93259971e/large.jpg
 https://assets.coolplaces.co.uk/images/9ac71e6f4ecf967d642ff49ec2192d7842beff69/large.jpg</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Off-Grid Holiday</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>https://www.offgrid-holiday.co.uk/</t>
         </is>
       </c>
     </row>
@@ -1452,6 +1552,16 @@
 https://assets.coolplaces.co.uk/images/e08f616cf6b850bd08044b9001623ec42c4ab631/large.jpg</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Once Upon a Fell</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>https://www.onceuponafell.co.uk/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1547,6 +1657,16 @@
 https://assets.coolplaces.co.uk/images/53e4ba34f1e7a83569bed3ded7db68f936538b1c/large.jpg</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/top-of-the-woods/</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1629,6 +1749,16 @@
 https://assets.coolplaces.co.uk/images/84baec28ba15cf6a4ea6ccdf79c9b2ee163f9c66/large.jpg</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Cairngorm Bothies</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>https://www.cairngormbothies.co.uk/</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1709,6 +1839,16 @@
 https://assets.coolplaces.co.uk/images/ffe3a079722475bba969ba4824f7f477bd93d15f/large.jpg
 https://assets.coolplaces.co.uk/images/7f534bcbe064ec4181d5d9dc1026b1ee6e1d7c5f/large.jpg
 https://assets.coolplaces.co.uk/images/ec6c2199aebdee3948f36a77009d518de8947234/large.jpg</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/den-by-the-stream/</t>
         </is>
       </c>
     </row>
@@ -1795,6 +1935,16 @@
 https://assets.coolplaces.co.uk/images/ef2a4835f4457e8353c788d10aea2e2ddafefe3a/large.jpg</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/england/herefordshire/the-fold/nova-dome</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1876,6 +2026,16 @@
 https://assets.coolplaces.co.uk/images/0dd1a2168dee8c5f48ef9d5d2f1d646fa4d3b063/large.jpg
 https://assets.coolplaces.co.uk/images/d3b71a2c9a87c047dd86ead2528f28aabfddb6f2/large.jpg
 https://assets.coolplaces.co.uk/images/237961712b2855066f1588998804eaa837ba64ec/large.jpg</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/england/herefordshire/the-fold/a-frame</t>
         </is>
       </c>
     </row>
@@ -1973,6 +2133,16 @@
 https://assets.coolplaces.co.uk/images/d137dd1ca23fc4341888731ffef26bce9e8b15e7/large.jpg</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/cabin-x-gpf/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2050,6 +2220,16 @@
 https://assets.coolplaces.co.uk/images/d586360b568a59b5228bd66a528f405d9b064fb9/large.jpg
 https://assets.coolplaces.co.uk/images/441352a1d0749a0801887ab04e959a7a130dee4d/large.jpg
 https://assets.coolplaces.co.uk/images/57ca5b68788e4188e3e781497aecef086b69bb45/large.jpg</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Cairngorm Lodges</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>https://www.cairngormlodges.co.uk/</t>
         </is>
       </c>
     </row>
@@ -2147,6 +2327,16 @@
 https://assets.coolplaces.co.uk/images/e56867cae1ac336c9792de32b9e84c19b48ff121/large.jpg</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Fernwood Glamping</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>https://www.fernwood-ringwood.co.uk/</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2242,6 +2432,16 @@
 https://assets.coolplaces.co.uk/images/e46842b4720bb0da8bc198cd867cb65dee4b3234/large.jpg</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/england/devon/wood-life-glamping</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2337,6 +2537,16 @@
 https://assets.coolplaces.co.uk/images/e57657a5052548b7cc11748ead197006056a3095/large.jpg</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/craighead-howfs/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2432,6 +2642,16 @@
 https://assets.coolplaces.co.uk/images/78f3803d8b320305aef9bbe2a24adaae7efdc977/large.jpg</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Kentmere Farm Pods</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>https://www.farmpods.co.uk/</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2527,6 +2747,16 @@
 https://assets.coolplaces.co.uk/images/976e3bcf7cf328a48a5c136fae474ec5313b8327/large.jpg</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/wales/carmarthenshire/under-starry-skies</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2607,6 +2837,16 @@
 https://assets.coolplaces.co.uk/images/e345366411e7483c1cd1b61c2644d1a5bb9a2ffc/large.jpg</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/albion-nights/</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2676,6 +2916,16 @@
 https://assets.coolplaces.co.uk/images/5409885bab456db734c477361deaf3e0f4beaf74/large.jpg
 https://assets.coolplaces.co.uk/images/12f7acab47b278246d2f130572628542c08af2d2/large.jpg
 https://assets.coolplaces.co.uk/images/3ad275af6296db02d64f10af3ff8bb4f53d9f80f/large.jpg</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Sykes Cottages</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>https://www.sykescottages.co.uk/cottage/Somerset-Aller-Fm/Beech-1147768.html</t>
         </is>
       </c>
     </row>
@@ -2767,6 +3017,16 @@
 https://assets.coolplaces.co.uk/images/99512294dc7e5f911ce1a37b0994ec07eaf49415/large.jpg</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Cotna Eco Retreat</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>https://cotna.co.uk/</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2837,6 +3097,16 @@
 https://assets.coolplaces.co.uk/images/699403ac16a657404815d249eed9dad1c90feb35/large.jpg
 https://assets.coolplaces.co.uk/images/3d3cc96d2ea6f550bf6cf116af07db31282b7473/large.jpg
 https://assets.coolplaces.co.uk/images/0675abc28fd7ca64871cfb08034051a9298b0be1/large.jpg</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Champing</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>https://champing.co.uk/church/penstrowed/</t>
         </is>
       </c>
     </row>
@@ -2919,6 +3189,16 @@
 https://assets.coolplaces.co.uk/images/850fd55e1ebd0be0e520526ea684fbebd86c319e/large.jpg
 https://assets.coolplaces.co.uk/images/419fec66ffa7f5c3c9ffb959ec92d667d70d0566/large.jpg
 https://assets.coolplaces.co.uk/images/9fb021e43b6ac9594abe5a024f9f2e4ad24ce5d5/large.jpg</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/england/herefordshire/the-fold/scandi-cabin</t>
         </is>
       </c>
     </row>
@@ -3016,6 +3296,16 @@
 https://assets.coolplaces.co.uk/images/50f31ceea0a41e01bbbe1ed648bdfeb5f74223bd/large.jpg</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Sloeberry Farm</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>https://sloeberryfarm.com/</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -3096,6 +3386,16 @@
 https://assets.coolplaces.co.uk/images/5130d0fd93d750f977e12dfdd34c7175111b1293/large.jpg
 https://assets.coolplaces.co.uk/images/24baa4ca674a94c2fd300103204e62ba519e3b0c/large.jpg
 https://assets.coolplaces.co.uk/images/227b74893a8617ffb7a36abf3ad916d4954a083f/large.jpg</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Berry Farm</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>https://stay.berryfarmprojects.org.uk</t>
         </is>
       </c>
     </row>
@@ -3179,6 +3479,16 @@
 https://assets.coolplaces.co.uk/images/bd8f52f6c6b27adb055fd18dcbe6d855dd2db428/large.jpg
 https://assets.coolplaces.co.uk/images/eae636a32d0a753d656dc7efc40aafb3daf15374/large.jpg
 https://assets.coolplaces.co.uk/images/334c5d43e8445eac46a4178cc5b5d242afed6ba5/large.jpg</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Wild Luxury</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>https://wildluxury.co.uk/</t>
         </is>
       </c>
     </row>
@@ -3266,6 +3576,16 @@
 https://assets.coolplaces.co.uk/images/e9d6da53bbb58796990815f5389b2efe83171d29/large.jpg</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/england/herefordshire/the-fold/the-treehouse</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3347,6 +3667,16 @@
 https://assets.coolplaces.co.uk/images/8890a1b97a7a461755c11d015b26721726587356/large.jpg
 https://assets.coolplaces.co.uk/images/88066d8be1bf992bc85fa78f0e00b3361b8d3e35/large.jpg
 https://assets.coolplaces.co.uk/images/ec206d8a33ad9fa57f1183d27cf58ce6071d4742/large.jpg</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Anglesey Shepherds Huts</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>https://angleseyshepherdshuts.org/</t>
         </is>
       </c>
     </row>
@@ -3444,6 +3774,16 @@
 https://assets.coolplaces.co.uk/images/d6555fb257fd5a05d4e0ee8e7fc256f92a4e517b/large.jpg</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Coolstays</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>https://www.coolstays.com/property/canvas-campfires/20591</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3515,6 +3855,16 @@
 https://assets.coolplaces.co.uk/images/a9343f34bac8fd76ff39cfd9bd4ade3c5e2ef133/large.jpg
 https://assets.coolplaces.co.uk/images/4caf68c98e68797cb5b390d6d9fdf2cd7de7fc13/large.jpg
 https://assets.coolplaces.co.uk/images/4661106e13ca6dbd542f5c85155ddff704d3f255/large.jpg</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Champing</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>https://champing.co.uk/church/langport-somerset-saints/</t>
         </is>
       </c>
     </row>
@@ -3595,6 +3945,16 @@
 https://assets.coolplaces.co.uk/images/9e27cf639450a3a1f507ba76331c32d0eb4397d9/large.jpg
 https://assets.coolplaces.co.uk/images/53909fb512431e064bc64d807f2acd89d80d124d/large.jpg
 https://assets.coolplaces.co.uk/images/ab9ffebf37420b23c6a56b846f024f50aa7f82bd/large.jpg</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Champing</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>https://champing.co.uk/church/laxfield-suffolk-champing-church/</t>
         </is>
       </c>
     </row>
@@ -3682,6 +4042,16 @@
 https://assets.coolplaces.co.uk/images/57f83665e9d0fd2210be72f479295282fa249eca/large.jpg
 https://assets.coolplaces.co.uk/images/e9728db27f9742cd16c7d97286a0993237ecdda8/large.jpg
 https://assets.coolplaces.co.uk/images/4774682195b54a62bfbf14809702c5bd0f02d564/large.jpg</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Choo Choo Moo</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>https://www.choochoomoo.com/</t>
         </is>
       </c>
     </row>
@@ -3779,6 +4149,16 @@
 https://assets.coolplaces.co.uk/images/c0c4a3e52853d196fc961cc04d2bee3dc6973836/large.jpg</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Canopy &amp; Stars</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>https://www.canopyandstars.co.uk/britain/england/shropshire/kinton</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3862,6 +4242,16 @@
 https://assets.coolplaces.co.uk/images/0abfb7d6f4c4fd9d46c5fe2c39ae51e5d5ce8a9e/large.jpg
 https://assets.coolplaces.co.uk/images/64a2bdff482e4f06dc9fc726a699c5c370db6939/large.jpg
 https://assets.coolplaces.co.uk/images/419d3bc3e809a86ab82c7cfea7fc5742b1af3091/large.jpg</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Coolstays</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>https://www.coolstays.com/property/lower-keats-glamping/18883</t>
         </is>
       </c>
     </row>
@@ -3956,6 +4346,16 @@
 https://assets.coolplaces.co.uk/images/e4b63a6b5fb831c3291e1c68a210845ad26ddd50/large.jpg</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Host Unusual</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>https://hostunusual.com/property/roulotte-retreat/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -4034,6 +4434,16 @@
 https://assets.coolplaces.co.uk/images/3d49e54890a5d4dd1318b1907a3d1c001d56ae0b/large.jpg</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Shillingridge Glamping</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>https://www.shillingridge.co.uk/lodges/lodge-availability</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -4102,6 +4512,16 @@
 https://assets.coolplaces.co.uk/images/6299f50339a3dd8dd705610f088da14a01ea52ed/large.jpg
 https://assets.coolplaces.co.uk/images/be2ed01b7da682b5dd798397e07eccfc8ba9a3a6/large.jpg
 https://assets.coolplaces.co.uk/images/31d589ba3187f6b923270335b2893e58896d8430/large.jpg</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Champing</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>https://champing.co.uk/church/arkengarthdale-north-yorkshire-st-marys/</t>
         </is>
       </c>
     </row>
@@ -4188,6 +4608,16 @@
 https://assets.coolplaces.co.uk/images/359ee8774ceb70d84936ad08cb5c97f0c0dcf640/large.jpg
 https://assets.coolplaces.co.uk/images/ef2e8dafce7f0755ba477e4d3576186652ddce65/large.jpg
 https://assets.coolplaces.co.uk/images/cb5fd75704e7220c287b353b21364a33415f0e17/large.jpg</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>The Original Hut Company</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>https://original-huts.co.uk/</t>
         </is>
       </c>
     </row>
@@ -4283,6 +4713,16 @@
 https://assets.coolplaces.co.uk/images/5c636cb477c3b1865874123d16e05351c6eaad12/large.jpg
 https://assets.coolplaces.co.uk/images/88897e5466e615a345db3b5be51c54fb5e5260ad/large.jpg
 https://assets.coolplaces.co.uk/images/d907370171d36252d0f28f84cb400d8c6a7a5ee8/large.jpg</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Wildings Holidays</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>https://wildingsholidays.co.uk/</t>
         </is>
       </c>
     </row>

</xml_diff>